<commit_message>
Added similarity_test.py for SSIM comparison of unlabelled and labelled images.
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Facultate\Disertatie\mainProject\pythonProject1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1481CCD3-DE29-4BE6-B933-46EB1A484452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A38A6E2-2036-4FD0-9D5F-296C1CF93A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{7C4DB224-D7E7-4677-B31E-EF3E3354B5EE}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" activeTab="1" xr2:uid="{7C4DB224-D7E7-4677-B31E-EF3E3354B5EE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="18.12.2025" sheetId="1" r:id="rId1"/>
+    <sheet name="16.12.2025" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="182">
   <si>
     <t>experiment_id</t>
   </si>
@@ -1036,12 +1037,150 @@
   <si>
     <t>copilot, chgpt - directii d ecerectare - ani, conditii</t>
   </si>
+  <si>
+    <t xml:space="preserve">
+  65   29    0    0   29   19
+   0  612    0    0    5    1
+   0   27  155    0   25    1
+   0    1    0  324    0    0
+   7   72   33    5  692   34
+   1   17    1    0   19  306
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+   8   42    1    1   32   58
+   2  555    0    1   40   20
+   4   36  115    0   28   25
+   0    1    0  322    1    1
+  20   75   19    5  645   79
+   0   10    1    1   10  322
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  55   30    0    0   31   26
+   0  610    0    0    7    1
+   0   25  156    0   24    3
+   0    1    0  324    0    0
+  10   76   30    6  681   40
+   0   18    1    0   15  310
+</t>
+  </si>
+  <si>
+    <t>2025-12-12 00:25:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ 118    3    0    0   17    4
+   2  612    0    0    3    1
+   0    2  165    0   41    0
+   1    0    0  321    3    0
+  14   15   18    3  769   24
+   1    3    0    0   17  323
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  64   31    2    0   30   15
+  10  580    2    0   21    5
+  10   26  141    0   26    5
+   0    0    1  319    4    1
+  49   66   29    4  663   32
+  29   14    1    0   13  287
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ 120    4    0    0   15    3
+   1  613    0    0    4    0
+   0    5  165    0   38    0
+   1    0    0  322    2    0
+  14   18   20    3  760   28
+   1    3    0    0   13  327
+</t>
+  </si>
+  <si>
+    <t>2025-12-12 21:38:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ 127    1    1    0   10    3
+   1  614    1    0    2    0
+   0    0  191    0   17    0
+   1    0    0  322    2    0
+  11   11   42    1  756   22
+   0    2    0    0   20  322
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  46   16    2    0   65   13
+  11  533    8    1   63    2
+   1    9  152    0   44    2
+   1    0    0  321    3    0
+  24   21   28    3  742   25
+  11    3    4    0   61  265
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ 124    1    0    0   13    4
+   0  614    1    0    3    0
+   0    0  191    0   17    0
+   1    0    0  323    1    0
+  11   12   35    1  764   20
+   0    2    0    0   17  325
+</t>
+  </si>
+  <si>
+    <t>2025-12-14 19:45:50</t>
+  </si>
+  <si>
+    <t>Pentru Cotraining - am antrenat doar o singura configuratie pentru fiecare dataset.</t>
+  </si>
+  <si>
+    <t>Rezultate antrenari modele individuale</t>
+  </si>
+  <si>
+    <t>test_gray_acc</t>
+  </si>
+  <si>
+    <t>gray_confusion_matrix</t>
+  </si>
+  <si>
+    <t>gray_pseudo_samples</t>
+  </si>
+  <si>
+    <t>final_gray_size</t>
+  </si>
+  <si>
+    <t>20% labeled</t>
+  </si>
+  <si>
+    <t>50% labeled</t>
+  </si>
+  <si>
+    <t>80% labeled</t>
+  </si>
+  <si>
+    <t>Model FFT / Test</t>
+  </si>
+  <si>
+    <t>Model Gray / Test</t>
+  </si>
+  <si>
+    <t>Model FFT / Validation</t>
+  </si>
+  <si>
+    <t>Model Gray / Validation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1058,6 +1197,20 @@
       <sz val="6"/>
       <color rgb="FFE3E3E3"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1127,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1157,11 +1310,30 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1272,7 +1444,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$2:$A$4</c:f>
+              <c:f>'18.12.2025'!$A$2:$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1289,7 +1461,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$2:$G$4</c:f>
+              <c:f>'18.12.2025'!$G$2:$G$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1326,7 +1498,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$2:$A$4</c:f>
+              <c:f>'18.12.2025'!$A$2:$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1343,7 +1515,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$2:$H$4</c:f>
+              <c:f>'18.12.2025'!$H$2:$H$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1380,7 +1552,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$2:$A$4</c:f>
+              <c:f>'18.12.2025'!$A$2:$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1397,7 +1569,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$2:$I$4</c:f>
+              <c:f>'18.12.2025'!$I$2:$I$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1706,7 +1878,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$2:$A$10</c:f>
+              <c:f>'18.12.2025'!$A$2:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
@@ -1741,7 +1913,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$2:$I$10</c:f>
+              <c:f>'18.12.2025'!$I$2:$I$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -2037,7 +2209,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$11:$A$19</c:f>
+              <c:f>'18.12.2025'!$A$11:$A$19</c:f>
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
@@ -2072,7 +2244,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$11:$I$19</c:f>
+              <c:f>'18.12.2025'!$I$11:$I$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -2368,7 +2540,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$20:$A$28</c:f>
+              <c:f>'18.12.2025'!$A$20:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
@@ -2403,7 +2575,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$20:$I$28</c:f>
+              <c:f>'18.12.2025'!$I$20:$I$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -2699,7 +2871,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$5:$A$7</c:f>
+              <c:f>'18.12.2025'!$A$5:$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -2716,7 +2888,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$5:$G$7</c:f>
+              <c:f>'18.12.2025'!$G$5:$G$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2753,7 +2925,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$5:$A$7</c:f>
+              <c:f>'18.12.2025'!$A$5:$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -2770,7 +2942,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$5:$H$7</c:f>
+              <c:f>'18.12.2025'!$H$5:$H$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -2807,7 +2979,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$5:$A$7</c:f>
+              <c:f>'18.12.2025'!$A$5:$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -2824,7 +2996,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$5:$I$7</c:f>
+              <c:f>'18.12.2025'!$I$5:$I$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3134,7 +3306,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$8:$A$10</c:f>
+              <c:f>'18.12.2025'!$A$8:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3151,7 +3323,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$8:$G$10</c:f>
+              <c:f>'18.12.2025'!$G$8:$G$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3188,7 +3360,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$8:$A$10</c:f>
+              <c:f>'18.12.2025'!$A$8:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3205,7 +3377,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$8:$H$10</c:f>
+              <c:f>'18.12.2025'!$H$8:$H$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3242,7 +3414,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$8:$A$10</c:f>
+              <c:f>'18.12.2025'!$A$8:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3259,7 +3431,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$8:$I$10</c:f>
+              <c:f>'18.12.2025'!$I$8:$I$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3569,7 +3741,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$11:$A$13</c:f>
+              <c:f>'18.12.2025'!$A$11:$A$13</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3586,7 +3758,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$11:$G$13</c:f>
+              <c:f>'18.12.2025'!$G$11:$G$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3623,7 +3795,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$11:$A$13</c:f>
+              <c:f>'18.12.2025'!$A$11:$A$13</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3640,7 +3812,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$11:$H$13</c:f>
+              <c:f>'18.12.2025'!$H$11:$H$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -3677,7 +3849,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$11:$A$13</c:f>
+              <c:f>'18.12.2025'!$A$11:$A$13</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -3694,7 +3866,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$11:$I$13</c:f>
+              <c:f>'18.12.2025'!$I$11:$I$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4003,7 +4175,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$14:$A$16</c:f>
+              <c:f>'18.12.2025'!$A$14:$A$16</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4020,7 +4192,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$14:$G$16</c:f>
+              <c:f>'18.12.2025'!$G$14:$G$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4057,7 +4229,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$14:$A$16</c:f>
+              <c:f>'18.12.2025'!$A$14:$A$16</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4074,7 +4246,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$14:$H$16</c:f>
+              <c:f>'18.12.2025'!$H$14:$H$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4111,7 +4283,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$14:$A$16</c:f>
+              <c:f>'18.12.2025'!$A$14:$A$16</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4128,7 +4300,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$14:$I$16</c:f>
+              <c:f>'18.12.2025'!$I$14:$I$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4437,7 +4609,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$17:$A$19</c:f>
+              <c:f>'18.12.2025'!$A$17:$A$19</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4454,7 +4626,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$17:$G$19</c:f>
+              <c:f>'18.12.2025'!$G$17:$G$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4491,7 +4663,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$17:$A$19</c:f>
+              <c:f>'18.12.2025'!$A$17:$A$19</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4508,7 +4680,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$17:$H$19</c:f>
+              <c:f>'18.12.2025'!$H$17:$H$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4545,7 +4717,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$17:$A$19</c:f>
+              <c:f>'18.12.2025'!$A$17:$A$19</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4562,7 +4734,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$17:$I$19</c:f>
+              <c:f>'18.12.2025'!$I$17:$I$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4872,7 +5044,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$20:$A$22</c:f>
+              <c:f>'18.12.2025'!$A$20:$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4889,7 +5061,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$20:$G$22</c:f>
+              <c:f>'18.12.2025'!$G$20:$G$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4926,7 +5098,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$20:$A$22</c:f>
+              <c:f>'18.12.2025'!$A$20:$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4943,7 +5115,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$20:$H$22</c:f>
+              <c:f>'18.12.2025'!$H$20:$H$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -4980,7 +5152,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$20:$A$22</c:f>
+              <c:f>'18.12.2025'!$A$20:$A$22</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -4997,7 +5169,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$20:$I$22</c:f>
+              <c:f>'18.12.2025'!$I$20:$I$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5306,7 +5478,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$23:$A$25</c:f>
+              <c:f>'18.12.2025'!$A$23:$A$25</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5323,7 +5495,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$23:$G$25</c:f>
+              <c:f>'18.12.2025'!$G$23:$G$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5360,7 +5532,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$23:$A$25</c:f>
+              <c:f>'18.12.2025'!$A$23:$A$25</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5377,7 +5549,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$23:$H$25</c:f>
+              <c:f>'18.12.2025'!$H$23:$H$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5414,7 +5586,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$23:$A$25</c:f>
+              <c:f>'18.12.2025'!$A$23:$A$25</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5431,7 +5603,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$23:$I$25</c:f>
+              <c:f>'18.12.2025'!$I$23:$I$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5768,7 +5940,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$26:$A$28</c:f>
+              <c:f>'18.12.2025'!$A$26:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5785,7 +5957,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$26:$G$28</c:f>
+              <c:f>'18.12.2025'!$G$26:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5822,7 +5994,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$26:$A$28</c:f>
+              <c:f>'18.12.2025'!$A$26:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5839,7 +6011,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$26:$H$28</c:f>
+              <c:f>'18.12.2025'!$H$26:$H$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -5876,7 +6048,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$26:$A$28</c:f>
+              <c:f>'18.12.2025'!$A$26:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -5893,7 +6065,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$26:$I$28</c:f>
+              <c:f>'18.12.2025'!$I$26:$I$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -13520,7 +13692,7 @@
       <c r="I2" s="3">
         <v>0.92459677419354802</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="12">
         <f>AVERAGE(I2:I10)</f>
         <v>0.93351254480286705</v>
       </c>
@@ -13583,7 +13755,7 @@
       <c r="I3" s="3">
         <v>0.94032258064516105</v>
       </c>
-      <c r="J3" s="11"/>
+      <c r="J3" s="12"/>
       <c r="K3" s="4" t="s">
         <v>26</v>
       </c>
@@ -13643,7 +13815,7 @@
       <c r="I4" s="3">
         <v>0.93064516129032204</v>
       </c>
-      <c r="J4" s="11"/>
+      <c r="J4" s="12"/>
       <c r="K4" s="4" t="s">
         <v>31</v>
       </c>
@@ -13703,7 +13875,7 @@
       <c r="I5" s="3">
         <v>0.93790322580645102</v>
       </c>
-      <c r="J5" s="11"/>
+      <c r="J5" s="12"/>
       <c r="K5" s="4" t="s">
         <v>36</v>
       </c>
@@ -13763,7 +13935,7 @@
       <c r="I6" s="3">
         <v>0.93225806451612903</v>
       </c>
-      <c r="J6" s="11"/>
+      <c r="J6" s="12"/>
       <c r="K6" s="4" t="s">
         <v>41</v>
       </c>
@@ -13823,7 +13995,7 @@
       <c r="I7" s="3">
         <v>0.93830645161290305</v>
       </c>
-      <c r="J7" s="11"/>
+      <c r="J7" s="12"/>
       <c r="K7" s="4" t="s">
         <v>46</v>
       </c>
@@ -13883,7 +14055,7 @@
       <c r="I8" s="3">
         <v>0.93991935483870903</v>
       </c>
-      <c r="J8" s="11"/>
+      <c r="J8" s="12"/>
       <c r="K8" s="4" t="s">
         <v>51</v>
       </c>
@@ -13943,7 +14115,7 @@
       <c r="I9" s="3">
         <v>0.93709677419354798</v>
       </c>
-      <c r="J9" s="11"/>
+      <c r="J9" s="12"/>
       <c r="K9" s="4" t="s">
         <v>56</v>
       </c>
@@ -14003,7 +14175,7 @@
       <c r="I10" s="3">
         <v>0.92056451612903201</v>
       </c>
-      <c r="J10" s="11"/>
+      <c r="J10" s="12"/>
       <c r="K10" s="4" t="s">
         <v>61</v>
       </c>
@@ -14063,7 +14235,7 @@
       <c r="I11" s="3">
         <v>0.90967741935483803</v>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="13">
         <f>AVERAGE(I11:I19)</f>
         <v>0.90869175627240095</v>
       </c>
@@ -14126,7 +14298,7 @@
       <c r="I12" s="3">
         <v>0.91774193548387095</v>
       </c>
-      <c r="J12" s="12"/>
+      <c r="J12" s="13"/>
       <c r="K12" s="4" t="s">
         <v>72</v>
       </c>
@@ -14186,7 +14358,7 @@
       <c r="I13" s="3">
         <v>0.87822580645161197</v>
       </c>
-      <c r="J13" s="12"/>
+      <c r="J13" s="13"/>
       <c r="K13" s="4" t="s">
         <v>72</v>
       </c>
@@ -14246,7 +14418,7 @@
       <c r="I14" s="3">
         <v>0.91370967741935405</v>
       </c>
-      <c r="J14" s="12"/>
+      <c r="J14" s="13"/>
       <c r="K14" s="4" t="s">
         <v>72</v>
       </c>
@@ -14306,7 +14478,7 @@
       <c r="I15" s="3">
         <v>0.912903225806451</v>
       </c>
-      <c r="J15" s="12"/>
+      <c r="J15" s="13"/>
       <c r="K15" s="4" t="s">
         <v>72</v>
       </c>
@@ -14366,7 +14538,7 @@
       <c r="I16" s="3">
         <v>0.92338709677419295</v>
       </c>
-      <c r="J16" s="12"/>
+      <c r="J16" s="13"/>
       <c r="K16" s="4" t="s">
         <v>72</v>
       </c>
@@ -14426,7 +14598,7 @@
       <c r="I17" s="3">
         <v>0.89274193548387004</v>
       </c>
-      <c r="J17" s="12"/>
+      <c r="J17" s="13"/>
       <c r="K17" s="4" t="s">
         <v>72</v>
       </c>
@@ -14486,7 +14658,7 @@
       <c r="I18" s="3">
         <v>0.91774193548387095</v>
       </c>
-      <c r="J18" s="12"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="4" t="s">
         <v>72</v>
       </c>
@@ -14546,7 +14718,7 @@
       <c r="I19" s="3">
         <v>0.91209677419354795</v>
       </c>
-      <c r="J19" s="12"/>
+      <c r="J19" s="13"/>
       <c r="K19" s="4" t="s">
         <v>101</v>
       </c>
@@ -14606,7 +14778,7 @@
       <c r="I20" s="3">
         <v>0.82741935483870899</v>
       </c>
-      <c r="J20" s="12">
+      <c r="J20" s="13">
         <f>AVERAGE(I20:I28)</f>
         <v>0.85703405017921108</v>
       </c>
@@ -14669,7 +14841,7 @@
       <c r="I21" s="3">
         <v>0.78830645161290303</v>
       </c>
-      <c r="J21" s="12"/>
+      <c r="J21" s="13"/>
       <c r="K21" s="4" t="s">
         <v>112</v>
       </c>
@@ -14729,7 +14901,7 @@
       <c r="I22" s="3">
         <v>0.84435483870967698</v>
       </c>
-      <c r="J22" s="12"/>
+      <c r="J22" s="13"/>
       <c r="K22" s="4" t="s">
         <v>117</v>
       </c>
@@ -14789,7 +14961,7 @@
       <c r="I23" s="3">
         <v>0.86532258064516099</v>
       </c>
-      <c r="J23" s="12"/>
+      <c r="J23" s="13"/>
       <c r="K23" s="4" t="s">
         <v>122</v>
       </c>
@@ -14849,7 +15021,7 @@
       <c r="I24" s="3">
         <v>0.87782258064516105</v>
       </c>
-      <c r="J24" s="12"/>
+      <c r="J24" s="13"/>
       <c r="K24" s="4" t="s">
         <v>127</v>
       </c>
@@ -14909,7 +15081,7 @@
       <c r="I25" s="3">
         <v>0.84798387096774197</v>
       </c>
-      <c r="J25" s="12"/>
+      <c r="J25" s="13"/>
       <c r="K25" s="4" t="s">
         <v>132</v>
       </c>
@@ -14969,7 +15141,7 @@
       <c r="I26" s="3">
         <v>0.89233870967741902</v>
       </c>
-      <c r="J26" s="12"/>
+      <c r="J26" s="13"/>
       <c r="K26" s="4" t="s">
         <v>137</v>
       </c>
@@ -15029,7 +15201,7 @@
       <c r="I27" s="3">
         <v>0.87379032258064504</v>
       </c>
-      <c r="J27" s="12"/>
+      <c r="J27" s="13"/>
       <c r="K27" s="4" t="s">
         <v>142</v>
       </c>
@@ -15089,7 +15261,7 @@
       <c r="I28" s="3">
         <v>0.89596774193548301</v>
       </c>
-      <c r="J28" s="12"/>
+      <c r="J28" s="13"/>
       <c r="K28" s="4" t="s">
         <v>147</v>
       </c>
@@ -15179,4 +15351,327 @@
   </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79FA2903-7A13-453F-A632-E06CB39D97BF}">
+  <dimension ref="A1:S13"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.69140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.07421875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.15234375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.3828125" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="18.53515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="19.53515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.23046875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.15234375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.07421875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.4609375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="17.69140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="116.6" x14ac:dyDescent="0.4">
+      <c r="A2" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="11">
+        <v>80</v>
+      </c>
+      <c r="D2" s="11">
+        <v>5</v>
+      </c>
+      <c r="E2" s="11">
+        <v>0.95</v>
+      </c>
+      <c r="F2" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="G2" s="17">
+        <v>0.86854838709677396</v>
+      </c>
+      <c r="H2" s="11">
+        <v>0.79314516129032198</v>
+      </c>
+      <c r="I2" s="11">
+        <v>0.86129032258064497</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="M2" s="11">
+        <v>6</v>
+      </c>
+      <c r="N2" s="11">
+        <v>3465</v>
+      </c>
+      <c r="O2" s="11">
+        <v>4401</v>
+      </c>
+      <c r="P2" s="11">
+        <v>7371</v>
+      </c>
+      <c r="Q2" s="11">
+        <v>2172</v>
+      </c>
+      <c r="R2" s="11">
+        <v>3108</v>
+      </c>
+      <c r="S2" s="17" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="116.6" x14ac:dyDescent="0.4">
+      <c r="A3" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="11">
+        <v>50</v>
+      </c>
+      <c r="D3" s="11">
+        <v>5</v>
+      </c>
+      <c r="E3" s="11">
+        <v>0.95</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="11">
+        <v>0.93064516129032204</v>
+      </c>
+      <c r="H3" s="11">
+        <v>0.82822580645161203</v>
+      </c>
+      <c r="I3" s="11">
+        <v>0.93024193548387102</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="M3" s="11">
+        <v>6</v>
+      </c>
+      <c r="N3" s="11">
+        <v>5548</v>
+      </c>
+      <c r="O3" s="11">
+        <v>6097</v>
+      </c>
+      <c r="P3" s="11">
+        <v>4866</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>1333</v>
+      </c>
+      <c r="R3" s="11">
+        <v>1882</v>
+      </c>
+      <c r="S3" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="116.6" x14ac:dyDescent="0.4">
+      <c r="A4" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="11">
+        <v>20</v>
+      </c>
+      <c r="D4" s="11">
+        <v>5</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0.95</v>
+      </c>
+      <c r="F4" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="G4" s="11">
+        <v>0.94032258064516105</v>
+      </c>
+      <c r="H4" s="11">
+        <v>0.83024193548387004</v>
+      </c>
+      <c r="I4" s="11">
+        <v>0.94395161290322505</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="M4" s="11">
+        <v>6</v>
+      </c>
+      <c r="N4" s="11">
+        <v>7074</v>
+      </c>
+      <c r="O4" s="11">
+        <v>6929</v>
+      </c>
+      <c r="P4" s="11">
+        <v>1946</v>
+      </c>
+      <c r="Q4" s="11">
+        <v>330</v>
+      </c>
+      <c r="R4" s="11">
+        <v>185</v>
+      </c>
+      <c r="S4" s="17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A6" s="14" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="B9" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>178</v>
+      </c>
+      <c r="B10">
+        <v>0.75890000000000002</v>
+      </c>
+      <c r="C10">
+        <v>0.78910000000000002</v>
+      </c>
+      <c r="D10">
+        <v>0.82179999999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11">
+        <v>0.73829999999999996</v>
+      </c>
+      <c r="C11">
+        <v>0.7944</v>
+      </c>
+      <c r="D11">
+        <v>0.83540000000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>181</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>